<commit_message>
fix(tender): reconcile Lot 5, Form C TCO baseline, editable compliance matrix, battery >=20kWh, and launch milestones
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
+++ b/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
@@ -585,10 +585,11 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Tender Ref: RFP-TELTECH-FWA-2026-001 | Author: OLIVER TUNGOL | Date: October 14, 2026</t>
-        </is>
-      </c>
-    </row>
+          <t>Tender Ref: RFP-TELTECH-FWA-2026-001 | Date: October 14, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -610,6 +611,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
@@ -1046,7 +1048,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>19" 3U/4U modular high-efficiency switchmode rectifier system; continuous rating &gt;= 6.0 kW @ -48V DC.</t>
+          <t>19" 3U/4U modular high-efficiency switchmode rectifier system; continuous rating &gt;= 12.0 kW @ -48V DC (4 x 3.0 kW modules in N+1 redundancy).</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr"/>
@@ -1065,7 +1067,7 @@
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Hot-swappable 2.0 kW or 3.0 kW modules in N+1 redundant configuration. Operating efficiency &gt;= 96.0%.</t>
+          <t>Hot-swappable 3.0 kW modules in N+1 redundant configuration (4x 3.0 kW modules total). Operating efficiency &gt;= 96.0%.</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr"/>
@@ -1103,7 +1105,7 @@
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Lithium Iron Phosphate (LiFePO4 / LFP) battery energy storage system: Sized to deliver at least 12.0 kWh usable energy to 3.0 kW DC continuous BTS load over 4.0 continuous hours without AC power, dimensioned for max 80% usable DoD and 80% end-of-life SoH retained capacity (min &gt;= 19.0 to 20.0 kWh nominal installed bank capacity, e.g., 4 x 48V 100 Ah modules or equivalent). Bidder shall submit formal load-autonomy calculation sheet, manufacturer discharge curves, and guarantee 4.0h autonomy at SAT.</t>
+          <t>Lithium Iron Phosphate (LiFePO4 / LFP) battery energy storage system: Sized to deliver at least 12.0 kWh usable energy to 3.0 kW DC continuous BTS load over 4.0 continuous hours without AC power, dimensioned for max 80% usable DoD and 80% end-of-life SoH retained capacity (minimum &gt;= 20.0 kWh nominal installed capacity, minimum 400 Ah to 450 Ah @ 48V, dimensioned via mandatory loss-based engineering calculation delivering 12.0 kWh net usable energy at 80% DoD and 80% EOL SoH). Bidder shall submit formal load-autonomy calculation sheet, manufacturer discharge curves, and guarantee 4.0h autonomy at SAT.</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr"/>
@@ -2183,7 +2185,7 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Indoor CPE: 230V AC / 12V DC external adapter (Philippine standard Type A/B plug). Outdoor CPE: 802.3at/af Power over Ethernet (PoE) injector included.</t>
+          <t>Indoor CPE: 230V AC / 12V DC external adapter (Philippine standard Type A/B plug). Outdoor CPE: 2.5GE-capable 802.3at/bt PoE power injector and 2.5GE WAN indoor gateway companion included.</t>
         </is>
       </c>
       <c r="D95" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
fix(commercial): de-duplicate Lot 1 & Lot 5 services, clarify 12kW installed/9kW firm N+1 rectifier, fix Lot 5 A2 & G14, and align Form C AMC basis
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
+++ b/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
@@ -1048,7 +1048,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>19" 3U/4U modular high-efficiency switchmode rectifier system; continuous rating &gt;= 12.0 kW @ -48V DC (4 x 3.0 kW modules in N+1 redundancy).</t>
+          <t>19" 3U/4U modular high-efficiency switchmode rectifier system; continuous rating &gt;= 12.0 kW total installed / 9.0 kW firm N+1 capacity @ -48V DC (4 x 3.0 kW modules: 3 active + 1 redundant standby).</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr"/>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Hot-swappable 3.0 kW modules in N+1 redundant configuration (4x 3.0 kW modules total). Operating efficiency &gt;= 96.0%.</t>
+          <t>Hot-swappable 3.0 kW modules in N+1 redundant configuration (4x 3.0 kW modules total, 3 active + 1 standby). Operating efficiency &gt;= 96.0%.</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr"/>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Lithium Iron Phosphate (LiFePO4 / LFP) battery energy storage system: Sized to deliver at least 12.0 kWh usable energy to 3.0 kW DC continuous BTS load over 4.0 continuous hours without AC power, dimensioned for max 80% usable DoD and 80% end-of-life SoH retained capacity (minimum &gt;= 20.0 kWh nominal installed capacity, minimum 400 Ah to 450 Ah @ 48V, dimensioned via mandatory loss-based engineering calculation delivering 12.0 kWh net usable energy at 80% DoD and 80% EOL SoH). Bidder shall submit formal load-autonomy calculation sheet, manufacturer discharge curves, and guarantee 4.0h autonomy at SAT.</t>
+          <t>Lithium Iron Phosphate (LiFePO4 / LFP) battery energy storage system: Sized to deliver at least 12.0 kWh usable energy to 3.0 kW DC continuous BTS load over 4.0 continuous hours without AC power, dimensioned for max 80% usable DoD and 80% end-of-life SoH retained capacity (minimum &gt;= 20.0 kWh nominal installed capacity is controlling; 400 Ah to 450 Ah is indicative, dimensioned via mandatory loss-based engineering calculation delivering 12.0 kWh net usable energy at 80% DoD and 80% EOL SoH). Bidder shall submit formal load-autonomy calculation sheet, manufacturer discharge curves, and guarantee 4.0h autonomy at SAT.</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
fix(compliance): align RAN-03 with dual-tier 60 MHz and 80 MHz channel bandwidths across all Appendix A deliverables and portal
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
+++ b/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Technical Compliance Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Compliance Scorecard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical Compliance Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compliance Scorecard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -697,7 +697,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Continuous 60 MHz channel bandwidth on a single carrier; software-configurable to 40 MHz / 50 MHz / 60 MHz.</t>
+          <t>Continuous 60 MHz (NCR / Meralco footprint, 162 RBs) and 80 MHz (Rest of Country / Provincial footprint, 217 RBs) single carrier; software-configurable to 40 MHz / 50 MHz / 60 MHz / 80 MHz.</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr"/>
@@ -870,7 +870,7 @@
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>Aggregated single-sector peak throughput &gt;= 450 Mbps in 60 MHz DL under 4:1 TDD frame configuration.</t>
+          <t>Aggregated single-sector peak throughput &gt;= 450 Mbps in 60 MHz DL (&gt;= 600 Mbps in 80 MHz DL) under 4:1 TDD frame configuration.</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr"/>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C86" s="16" t="inlineStr">
         <is>
-          <t>Native Band n50 (1432 – 1517 MHz, 60 MHz channel bandwidth) plus fallback sub-6 GHz bands (n1, n3, n7, n28, n41, n77, n78).</t>
+          <t>Native Band n50 (1432 – 1517 MHz, supporting 60 MHz and 80 MHz channel bandwidths) plus fallback sub-6 GHz bands (n1, n3, n7, n28, n41, n77, n78).</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(clarifications): publish Master Register (Q001-Q100) and RAN-21 RF conformance specs
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
+++ b/RFP_Tender_Package/02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +67,23 @@
       <color rgb="001B365D"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000A192F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E293B"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -100,7 +117,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -136,11 +153,69 @@
         <color rgb="0086EFAC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -193,6 +268,23 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -558,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -589,7 +681,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -611,7 +702,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
@@ -1028,1187 +1118,1171 @@
       <c r="D30" s="12" t="inlineStr"/>
       <c r="E30" s="13" t="inlineStr"/>
     </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="31" ht="110" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>RAN-21</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>RF Conformance &amp; Out-of-Band Emission Testing</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>Certified third-party or OEM factory laboratory test reports under 3GPP TS 38.141-1 (Conducted) and TS 38.141-2 (Radiated) demonstrating:
+1. Spectrum Emission Mask (SEM) compliance at maximum rated conducted output power (+55 dBm / 320W per sector);
+2. Adjacent Channel Leakage Ratio (ACLR &gt;= 45 dB) into the adjacent 1432.0–1457.0 MHz NPN band;
+3. Operating Band Unwanted Emissions (OBUE) high-resolution spectral mask plots across 1517.0–1559.0 MHz verifying &lt;= -30 dBm/MHz out-of-band emissions above 1518.0 MHz for MSS satellite protection pursuant to ITU-R M.2159-0, WRC-15 Resolution 223, and NTC MC No. 006-11-2025;
+4. Spurious emissions across out-of-band ranges;
+5. Explicit manufacturer declaration of any required transmitter power de-rating (in dB) or external high-Q cavity bandpass filtering needed to achieve boundary compliance at maximum rated power, including quantified coverage impacts on the link budget.</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="n"/>
+      <c r="E31" s="26" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>SECTION 2: POWER SYSTEMS &amp; PASSIVE SITE INFRASTRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>PWR-01</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>DC Power Plant</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>19" 3U/4U modular high-efficiency switchmode rectifier system; continuous rating &gt;= 12.0 kW total installed / 9.0 kW firm N+1 capacity @ -48V DC (4 x 3.0 kW modules: 3 active + 1 redundant standby).</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr"/>
-      <c r="E32" s="13" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>PWR-02</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="inlineStr">
-        <is>
-          <t>Rectifier Modules</t>
-        </is>
-      </c>
-      <c r="C33" s="16" t="inlineStr">
-        <is>
-          <t>Hot-swappable 3.0 kW modules in N+1 redundant configuration (4x 3.0 kW modules total, 3 active + 1 standby). Operating efficiency &gt;= 96.0%.</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr"/>
       <c r="E33" s="13" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>PWR-03</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Input Voltage Range</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>Wide AC input operating range: 85V AC to 300V AC nominal single phase (230V, 60 Hz), withstanding rural grid fluctuations.</t>
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>PWR-02</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Rectifier Modules</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Hot-swappable 3.0 kW modules in N+1 redundant configuration (4x 3.0 kW modules total, 3 active + 1 standby). Operating efficiency &gt;= 96.0%.</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr"/>
       <c r="E34" s="13" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>PWR-04</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="inlineStr">
-        <is>
-          <t>Lithium Battery (BESS)</t>
-        </is>
-      </c>
-      <c r="C35" s="16" t="inlineStr">
-        <is>
-          <t>Lithium Iron Phosphate (LiFePO4 / LFP) battery energy storage system: Sized to deliver at least 12.0 kWh usable energy to 3.0 kW DC continuous BTS load over 4.0 continuous hours without AC power, dimensioned for max 80% usable DoD and 80% end-of-life SoH retained capacity (minimum &gt;= 20.0 kWh nominal installed capacity is controlling; 400 Ah to 450 Ah is indicative, dimensioned via mandatory loss-based engineering calculation delivering 12.0 kWh net usable energy at 80% DoD and 80% EOL SoH). Bidder shall submit formal load-autonomy calculation sheet, manufacturer discharge curves, and guarantee 4.0h autonomy at SAT.</t>
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>PWR-03</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Input Voltage Range</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Wide AC input operating range: 85V AC to 300V AC nominal single phase (230V, 60 Hz), withstanding rural grid fluctuations.</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr"/>
       <c r="E35" s="13" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>PWR-05</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Battery Autonomy</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Guaranteed &gt;= 4.0 hours continuous operation at 3.0 kW continuous BTS load without AC utility input, verified by full discharge test at site acceptance.</t>
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>PWR-04</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>Lithium Battery (BESS)</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Lithium Iron Phosphate (LiFePO4 / LFP) battery energy storage system: Sized to deliver at least 12.0 kWh usable energy to 3.0 kW DC continuous BTS load over 4.0 continuous hours without AC power, dimensioned for max 80% usable DoD and 80% end-of-life SoH retained capacity (minimum &gt;= 20.0 kWh nominal installed capacity is controlling; 400 Ah to 450 Ah is indicative, dimensioned via mandatory loss-based engineering calculation delivering 12.0 kWh net usable energy at 80% DoD and 80% EOL SoH). Bidder shall submit formal load-autonomy calculation sheet, manufacturer discharge curves, and guarantee 4.0h autonomy at SAT.</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr"/>
       <c r="E36" s="13" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>PWR-06</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>Battery Cycle Life</t>
-        </is>
-      </c>
-      <c r="C37" s="16" t="inlineStr">
-        <is>
-          <t>&gt;= 4,000 cycles at 80% Depth of Discharge (DoD) at +25°C; built-in intelligent Battery Management System (BMS).</t>
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>PWR-05</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Battery Autonomy</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Guaranteed &gt;= 4.0 hours continuous operation at 3.0 kW continuous BTS load without AC utility input, verified by full discharge test at site acceptance.</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr"/>
       <c r="E37" s="13" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="inlineStr">
-        <is>
-          <t>PWR-07</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Standby Genset</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="inlineStr">
-        <is>
-          <t>For Greenfield (Class T4) sites: 15 kVA / 12 kW prime, 230V, 60 Hz diesel generator in sound-attenuated weatherproof canopy (&lt;68dBA @ 7m).</t>
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>PWR-06</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>Battery Cycle Life</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>&gt;= 4,000 cycles at 80% Depth of Discharge (DoD) at +25°C; built-in intelligent Battery Management System (BMS).</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr"/>
       <c r="E38" s="13" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>PWR-08</t>
-        </is>
-      </c>
-      <c r="B39" s="15" t="inlineStr">
-        <is>
-          <t>Fuel Autonomy</t>
-        </is>
-      </c>
-      <c r="C39" s="16" t="inlineStr">
-        <is>
-          <t>Integrated sub-base fuel tank with minimum 500L–1,000L capacity providing &gt;= 72hours continuous runtime under full load.</t>
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>PWR-07</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Standby Genset</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>For Greenfield (Class T4) sites: 15 kVA / 12 kW prime, 230V, 60 Hz diesel generator in sound-attenuated weatherproof canopy (&lt;68dBA @ 7m).</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr"/>
       <c r="E39" s="13" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>PWR-09</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Automatic Transfer (ATS)</t>
-        </is>
-      </c>
-      <c r="C40" s="11" t="inlineStr">
-        <is>
-          <t>Microprocessor-controlled ATS with 4-pole motorized breaker and mechanical interlock, transferring power within 30 seconds of grid failure.</t>
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>PWR-08</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>Fuel Autonomy</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Integrated sub-base fuel tank with minimum 500L–1,000L capacity providing &gt;= 72hours continuous runtime under full load.</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr"/>
       <c r="E40" s="13" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>PWR-10</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>Surge Protection</t>
-        </is>
-      </c>
-      <c r="C41" s="16" t="inlineStr">
-        <is>
-          <t>Coordinated SPD Type 1+2 on AC input (&gt;= 40kA) and DC distribution busbar (&gt;= 20kA).</t>
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>PWR-09</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Automatic Transfer (ATS)</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Microprocessor-controlled ATS with 4-pole motorized breaker and mechanical interlock, transferring power within 30 seconds of grid failure.</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr"/>
       <c r="E41" s="13" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>PWR-11</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>TowerCo Tap-Off Kit</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>Standardized co-location DC tap box with integrated Class 1.0 revenue-grade kWh energy meter and RS485/Modbus telemetry.</t>
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>PWR-10</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>Surge Protection</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Coordinated SPD Type 1+2 on AC input (&gt;= 40kA) and DC distribution busbar (&gt;= 20kA).</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr"/>
       <c r="E42" s="13" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="inlineStr">
-        <is>
-          <t>PWR-12</t>
-        </is>
-      </c>
-      <c r="B43" s="15" t="inlineStr">
-        <is>
-          <t>Grounding &amp; Lightning</t>
-        </is>
-      </c>
-      <c r="C43" s="16" t="inlineStr">
-        <is>
-          <t>Comprehensive grounding system achieving &lt;= 5.0 Ohms earth electrode resistance; copper busbars and copper-clad steel ground rods.</t>
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>PWR-11</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>TowerCo Tap-Off Kit</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>Standardized co-location DC tap box with integrated Class 1.0 revenue-grade kWh energy meter and RS485/Modbus telemetry.</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr"/>
       <c r="E43" s="13" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>PWR-12</t>
+        </is>
+      </c>
+      <c r="B44" s="27" t="n"/>
+      <c r="C44" s="27" t="n"/>
+      <c r="D44" s="27" t="n"/>
+      <c r="E44" s="28" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>SECTION 3: 5G CORE NETWORK (5GC SA) &amp; DATACENTER INFRASTRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>5GC-01</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>Architecture</t>
         </is>
       </c>
-      <c r="C45" s="11" t="inlineStr">
+      <c r="C46" s="11" t="inlineStr">
         <is>
           <t>Cloud-native, containerized microservices 5G Standalone (5GC SA) compliant with 3GPP Release 16/17 Service-Based Architecture (SBA).</t>
-        </is>
-      </c>
-      <c r="D45" s="12" t="inlineStr"/>
-      <c r="E45" s="13" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="14" t="inlineStr">
-        <is>
-          <t>5GC-02</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="inlineStr">
-        <is>
-          <t>Network Functions</t>
-        </is>
-      </c>
-      <c r="C46" s="16" t="inlineStr">
-        <is>
-          <t>Full NF suite: AMF, SMF, UPF, PCF, UDM, UDR, AUSF, NRF, NSSF, NEF, CHF, and SEPP.</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr"/>
       <c r="E46" s="13" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="inlineStr">
-        <is>
-          <t>5GC-03</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>Subscriber Sizing</t>
-        </is>
-      </c>
-      <c r="C47" s="11" t="inlineStr">
-        <is>
-          <t>Day-1 licensed capacity: 1,000,000 registered FWA subscribers. Scalable in 500k increments up to 3,000,000 subscribers.</t>
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>5GC-02</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Network Functions</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Full NF suite: AMF, SMF, UPF, PCF, UDM, UDR, AUSF, NRF, NSSF, NEF, CHF, and SEPP.</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr"/>
       <c r="E47" s="13" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="inlineStr">
-        <is>
-          <t>5GC-04</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="inlineStr">
-        <is>
-          <t>Geo-Redundancy</t>
-        </is>
-      </c>
-      <c r="C48" s="16" t="inlineStr">
-        <is>
-          <t>Active-Active geo-redundant dual-datacenter deployment (Metro Manila Primary DC and Clark Pampanga DR DC).</t>
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>5GC-03</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Subscriber Sizing</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Day-1 licensed capacity: 1,000,000 registered FWA subscribers. Scalable in 500k increments up to 3,000,000 subscribers.</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr"/>
       <c r="E48" s="13" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="9" t="inlineStr">
-        <is>
-          <t>5GC-05</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Session-Preserving Failover</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>Automatic subscriber session continuity (zero session loss across UDR/UDM and SMF clusters) and automated user-plane traffic restoration &lt;= 30 seconds during datacenter failure or scheduled DR drill.</t>
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>5GC-04</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>Geo-Redundancy</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Active-Active geo-redundant dual-datacenter deployment (Metro Manila Primary DC and Clark Pampanga DR DC).</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr"/>
       <c r="E49" s="13" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="inlineStr">
-        <is>
-          <t>5GC-06</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>UPF Throughput</t>
-        </is>
-      </c>
-      <c r="C50" s="16" t="inlineStr">
-        <is>
-          <t>UPF dimensioned for &gt;= 80 Gbps usable wire-speed throughput per 2U dual-socket compute node with DPDK and SR-IOV acceleration.</t>
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>5GC-05</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>Session-Preserving Failover</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Automatic subscriber session continuity (zero session loss across UDR/UDM and SMF clusters) and automated user-plane traffic restoration &lt;= 30 seconds during datacenter failure or scheduled DR drill.</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr"/>
       <c r="E50" s="13" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>5GC-07</t>
-        </is>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>Carrier-Grade NAT</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>Integrated or inline CG-NAT supporting deterministic port allocation, logging per NTC legal intercept mandate, and 10:1 to 16:1 subscriber ratio.</t>
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>5GC-06</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>UPF Throughput</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>UPF dimensioned for &gt;= 80 Gbps usable wire-speed throughput per 2U dual-socket compute node with DPDK and SR-IOV acceleration.</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr"/>
       <c r="E51" s="13" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="14" t="inlineStr">
-        <is>
-          <t>5GC-08</t>
-        </is>
-      </c>
-      <c r="B52" s="15" t="inlineStr">
-        <is>
-          <t>Deep Packet Inspection</t>
-        </is>
-      </c>
-      <c r="C52" s="16" t="inlineStr">
-        <is>
-          <t>Embedded DPI capable of Layer-7 application recognition, speed throttling per subscriber tariff tier, and fair-use policy enforcement.</t>
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>5GC-07</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Carrier-Grade NAT</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>Integrated or inline CG-NAT supporting deterministic port allocation, logging per NTC legal intercept mandate, and 10:1 to 16:1 subscriber ratio.</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr"/>
       <c r="E52" s="13" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="inlineStr">
-        <is>
-          <t>5GC-09</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="inlineStr">
-        <is>
-          <t>QoS &amp; Slicing</t>
-        </is>
-      </c>
-      <c r="C53" s="11" t="inlineStr">
-        <is>
-          <t>5G QoS Flow mapping (5QI 1, 2, 7, 8, 9) and Network Slicing (S-NSSAI) separating consumer FWA, SME enterprise, and management traffic.</t>
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>5GC-08</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>Deep Packet Inspection</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>Embedded DPI capable of Layer-7 application recognition, speed throttling per subscriber tariff tier, and fair-use policy enforcement.</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr"/>
       <c r="E53" s="13" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
-        <is>
-          <t>5GC-10</t>
-        </is>
-      </c>
-      <c r="B54" s="15" t="inlineStr">
-        <is>
-          <t>Datacenter Compute</t>
-        </is>
-      </c>
-      <c r="C54" s="16" t="inlineStr">
-        <is>
-          <t>Enterprise 2U server nodes (Dual Intel Xeon Gold / AMD EPYC, 512GB RAM, redundant NVMe enterprise SSDs, dual 100GE NICs).</t>
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>5GC-09</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>QoS &amp; Slicing</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>5G QoS Flow mapping (5QI 1, 2, 7, 8, 9) and Network Slicing (S-NSSAI) separating consumer FWA, SME enterprise, and management traffic.</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr"/>
       <c r="E54" s="13" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
-        <is>
-          <t>5GC-11</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>Datacenter Fabric</t>
-        </is>
-      </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>Leaf-spine datacenter networking architecture (32 x 100GE spine switches, 48 x 25GE + 6 x 100GE leaf switches) with EVPN-VXLAN.</t>
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>5GC-10</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Datacenter Compute</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Enterprise 2U server nodes (Dual Intel Xeon Gold / AMD EPYC, 512GB RAM, redundant NVMe enterprise SSDs, dual 100GE NICs).</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr"/>
       <c r="E55" s="13" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>5GC-12</t>
-        </is>
-      </c>
-      <c r="B56" s="15" t="inlineStr">
-        <is>
-          <t>Security &amp; Scrubbing</t>
-        </is>
-      </c>
-      <c r="C56" s="16" t="inlineStr">
-        <is>
-          <t>Redundant carrier-grade perimeter next-generation firewalls (&gt;= 100 Gbps throughput) and inline anti-DDoS scrubbing appliances.</t>
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>5GC-11</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Datacenter Fabric</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Leaf-spine datacenter networking architecture (32 x 100GE spine switches, 48 x 25GE + 6 x 100GE leaf switches) with EVPN-VXLAN.</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr"/>
       <c r="E56" s="13" t="inlineStr"/>
     </row>
     <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>5GC-12</t>
+        </is>
+      </c>
+      <c r="B57" s="27" t="n"/>
+      <c r="C57" s="27" t="n"/>
+      <c r="D57" s="27" t="n"/>
+      <c r="E57" s="28" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
         <is>
           <t>BSS-01</t>
         </is>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B59" s="10" t="inlineStr">
         <is>
           <t>Product Catalog &amp; Tariffs</t>
         </is>
       </c>
-      <c r="C58" s="11" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>Configurable telecom product catalog supporting 4 consumer FWA plans (₱599, ₱799, ₱999, ₱1,299), SME tiers, and flexible speed-cap policies.</t>
-        </is>
-      </c>
-      <c r="D58" s="12" t="inlineStr"/>
-      <c r="E58" s="13" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="14" t="inlineStr">
-        <is>
-          <t>BSS-02</t>
-        </is>
-      </c>
-      <c r="B59" s="15" t="inlineStr">
-        <is>
-          <t>Prepaid Charging (CHF)</t>
-        </is>
-      </c>
-      <c r="C59" s="16" t="inlineStr">
-        <is>
-          <t>Real-time convergent charging system (CCS/CHF) integrated via 3GPP Nchf/Diameter Ro, supporting real-time balance rating and session cutoff.</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr"/>
       <c r="E59" s="13" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>BSS-03</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>Omnichannel Payments</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Native REST API integration with Philippine payment gateways: GCash, Maya (PayMaya), 7-Eleven CLiQQ OTC, Bayad Center, and QR Ph.</t>
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>BSS-02</t>
+        </is>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>Prepaid Charging (CHF)</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>Real-time convergent charging system (CCS/CHF) integrated via 3GPP Nchf/Diameter Ro, supporting real-time balance rating and session cutoff.</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr"/>
       <c r="E60" s="13" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="inlineStr">
-        <is>
-          <t>BSS-04</t>
-        </is>
-      </c>
-      <c r="B61" s="15" t="inlineStr">
-        <is>
-          <t>Subscriber Portal &amp; App</t>
-        </is>
-      </c>
-      <c r="C61" s="16" t="inlineStr">
-        <is>
-          <t>Native Android/iOS subscriber self-care mobile app and responsive web portal for balance checking, online top-up, and speed-test diagnostics.</t>
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>BSS-03</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>Omnichannel Payments</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>Native REST API integration with Philippine payment gateways: GCash, Maya (PayMaya), 7-Eleven CLiQQ OTC, Bayad Center, and QR Ph.</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr"/>
       <c r="E61" s="13" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OSS-01</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>Field Force App (FMS)</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Mobile app for field technicians: Real-time work-order dispatch, turn-by-turn navigation, barcode/QR scan of CPE serials, and digital e-signature.</t>
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>BSS-04</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>Subscriber Portal &amp; App</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Native Android/iOS subscriber self-care mobile app and responsive web portal for balance checking, online top-up, and speed-test diagnostics.</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr"/>
       <c r="E62" s="13" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="inlineStr">
-        <is>
-          <t>OSS-02</t>
-        </is>
-      </c>
-      <c r="B63" s="15" t="inlineStr">
-        <is>
-          <t>RF Signal Verification</t>
-        </is>
-      </c>
-      <c r="C63" s="16" t="inlineStr">
-        <is>
-          <t>Mobile field tool must perform live outdoor RF signal validation (RSRP &gt;= -95 dBm, SINR &gt;= 10 dB) before allowing install closure.</t>
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>OSS-01</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Field Force App (FMS)</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>Mobile app for field technicians: Real-time work-order dispatch, turn-by-turn navigation, barcode/QR scan of CPE serials, and digital e-signature.</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr"/>
       <c r="E63" s="13" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>OSS-03</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>Dispatch Throughput</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>Algorithmic dispatch engine capable of dynamically optimizing and dispatching &gt;= 3,500 installation and maintenance work orders daily.</t>
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>OSS-02</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>RF Signal Verification</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Mobile field tool must perform live outdoor RF signal validation (RSRP &gt;= -95 dBm, SINR &gt;= 10 dB) before allowing install closure.</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr"/>
       <c r="E64" s="13" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>OSS-04</t>
-        </is>
-      </c>
-      <c r="B65" s="15" t="inlineStr">
-        <is>
-          <t>CPE Inventory &amp; WMS</t>
-        </is>
-      </c>
-      <c r="C65" s="16" t="inlineStr">
-        <is>
-          <t>Serialized lifecycle tracking of CPE hardware across central warehouse, technician vehicle float, active subscriber homes, and repossession.</t>
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>OSS-03</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>Dispatch Throughput</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>Algorithmic dispatch engine capable of dynamically optimizing and dispatching &gt;= 3,500 installation and maintenance work orders daily.</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr"/>
       <c r="E65" s="13" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="inlineStr">
-        <is>
-          <t>OSS-05</t>
-        </is>
-      </c>
-      <c r="B66" s="10" t="inlineStr">
-        <is>
-          <t>Reverse Logistics</t>
-        </is>
-      </c>
-      <c r="C66" s="11" t="inlineStr">
-        <is>
-          <t>Reverse logistics workflow tracking recovered churned CPEs through testing, factory reset, cleaning, re-boxing, and return to stock (&gt;= 70% target).</t>
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>OSS-04</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>CPE Inventory &amp; WMS</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Serialized lifecycle tracking of CPE hardware across central warehouse, technician vehicle float, active subscriber homes, and repossession.</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr"/>
       <c r="E66" s="13" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="14" t="inlineStr">
-        <is>
-          <t>OSS-06</t>
-        </is>
-      </c>
-      <c r="B67" s="15" t="inlineStr">
-        <is>
-          <t>Fault &amp; Performance OSS</t>
-        </is>
-      </c>
-      <c r="C67" s="16" t="inlineStr">
-        <is>
-          <t>Unified multi-vendor EMS/NMS monitoring 5,000 RAN sites, transmission links, and 5G Core with automated RCA and alarm correlation.</t>
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>OSS-05</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>Reverse Logistics</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>Reverse logistics workflow tracking recovered churned CPEs through testing, factory reset, cleaning, re-boxing, and return to stock (&gt;= 70% target).</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr"/>
       <c r="E67" s="13" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="inlineStr">
-        <is>
-          <t>OSS-07</t>
-        </is>
-      </c>
-      <c r="B68" s="10" t="inlineStr">
-        <is>
-          <t>Regulatory Compliance</t>
-        </is>
-      </c>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t>Automated generation of quarterly NTC Quality of Service (QoS) and broadband speed performance audit reports.</t>
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>OSS-06</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>Fault &amp; Performance OSS</t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>Unified multi-vendor EMS/NMS monitoring 5,000 RAN sites, transmission links, and 5G Core with automated RCA and alarm correlation.</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr"/>
       <c r="E68" s="13" t="inlineStr"/>
     </row>
     <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>OSS-07</t>
+        </is>
+      </c>
+      <c r="B69" s="27" t="n"/>
+      <c r="C69" s="27" t="n"/>
+      <c r="D69" s="27" t="n"/>
+      <c r="E69" s="28" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>SECTION 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="14" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
         <is>
           <t>RFP-01</t>
         </is>
       </c>
-      <c r="B70" s="15" t="inlineStr">
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>Planning Tool</t>
         </is>
       </c>
-      <c r="C70" s="16" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
         <is>
           <t>Carrier-grade RF planning tool (Atoll, Asset, Planet) with high-resolution digital terrain and clutter data (&lt;= 5m resolution).</t>
-        </is>
-      </c>
-      <c r="D70" s="12" t="inlineStr"/>
-      <c r="E70" s="13" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="9" t="inlineStr">
-        <is>
-          <t>RFP-02</t>
-        </is>
-      </c>
-      <c r="B71" s="10" t="inlineStr">
-        <is>
-          <t>Propagation Model</t>
-        </is>
-      </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>Calibrated Band n50 (1.5 GHz) 3D ray-tracing / standard propagation model calibrated against local Philippine terrain clutter.</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr"/>
       <c r="E71" s="13" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="14" t="inlineStr">
-        <is>
-          <t>RFP-03</t>
-        </is>
-      </c>
-      <c r="B72" s="15" t="inlineStr">
-        <is>
-          <t>Nominal Siting &amp; Audit</t>
-        </is>
-      </c>
-      <c r="C72" s="16" t="inlineStr">
-        <is>
-          <t>Siting validation against 13,746 tower inventory and Converge fiber network backbone routes (subject to verification on the ground); production of candidate search rings.</t>
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>RFP-02</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>Propagation Model</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>Calibrated Band n50 (1.5 GHz) 3D ray-tracing / standard propagation model calibrated against local Philippine terrain clutter.</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr"/>
       <c r="E72" s="13" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="9" t="inlineStr">
-        <is>
-          <t>RFP-04</t>
-        </is>
-      </c>
-      <c r="B73" s="10" t="inlineStr">
-        <is>
-          <t>Technical Site Survey</t>
-        </is>
-      </c>
-      <c r="C73" s="11" t="inlineStr">
-        <is>
-          <t>Comprehensive TSSR per site including tower structural load audit, wind-load calculation, panoramic drone photography (360°), and power audit.</t>
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>RFP-03</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>Nominal Siting &amp; Audit</t>
+        </is>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>Siting validation against 13,746 tower inventory and Converge fiber network backbone routes (subject to verification on the ground); production of candidate search rings.</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr"/>
       <c r="E73" s="13" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="14" t="inlineStr">
-        <is>
-          <t>RFP-05</t>
-        </is>
-      </c>
-      <c r="B74" s="15" t="inlineStr">
-        <is>
-          <t>Coverage Target</t>
-        </is>
-      </c>
-      <c r="C74" s="16" t="inlineStr">
-        <is>
-          <t>Guaranteed outdoor RSRP &gt;= -95 dBm and SINR &gt;= 10 dB across &gt;= 90% of residential settlement footprint in target barangay.</t>
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>RFP-04</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Technical Site Survey</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>Comprehensive TSSR per site including tower structural load audit, wind-load calculation, panoramic drone photography (360°), and power audit.</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr"/>
       <c r="E74" s="13" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="inlineStr">
-        <is>
-          <t>RFP-06</t>
-        </is>
-      </c>
-      <c r="B75" s="10" t="inlineStr">
-        <is>
-          <t>Single Site Acceptance</t>
-        </is>
-      </c>
-      <c r="C75" s="11" t="inlineStr">
-        <is>
-          <t>Single Site Verification (SSV) stationary and drive tests verifying sector radiation, antenna RET, PCI, TAC, and max throughput.</t>
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>RFP-05</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>Coverage Target</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Guaranteed outdoor RSRP &gt;= -95 dBm and SINR &gt;= 10 dB across &gt;= 90% of residential settlement footprint in target barangay.</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr"/>
       <c r="E75" s="13" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="14" t="inlineStr">
-        <is>
-          <t>RFP-07</t>
-        </is>
-      </c>
-      <c r="B76" s="15" t="inlineStr">
-        <is>
-          <t>Cluster Tuning</t>
-        </is>
-      </c>
-      <c r="C76" s="16" t="inlineStr">
-        <is>
-          <t>Cluster optimization across 10–20 site clusters: Interference analysis, tilt/azimuth physical optimization, handover parameter tuning.</t>
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>RFP-06</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>Single Site Acceptance</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>Single Site Verification (SSV) stationary and drive tests verifying sector radiation, antenna RET, PCI, TAC, and max throughput.</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr"/>
       <c r="E76" s="13" t="inlineStr"/>
     </row>
     <row r="77" ht="22" customHeight="1">
-      <c r="A77" s="8" t="inlineStr">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>RFP-07</t>
+        </is>
+      </c>
+      <c r="B77" s="27" t="n"/>
+      <c r="C77" s="27" t="n"/>
+      <c r="D77" s="27" t="n"/>
+      <c r="E77" s="28" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
         <is>
           <t>SECTION 6: MANAGED SERVICES &amp; 24/7 NETWORK OPERATIONS (MS)</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="9" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="9" t="inlineStr">
         <is>
           <t>MS-01</t>
         </is>
       </c>
-      <c r="B78" s="10" t="inlineStr">
+      <c r="B79" s="10" t="inlineStr">
         <is>
           <t>24/7 Tier-2/Tier-3 NOC</t>
         </is>
       </c>
-      <c r="C78" s="11" t="inlineStr">
+      <c r="C79" s="11" t="inlineStr">
         <is>
           <t>Continuous 24/7/365 active monitoring, incident triage, alarm dispatch, and escalation management across all network domains.</t>
-        </is>
-      </c>
-      <c r="D78" s="12" t="inlineStr"/>
-      <c r="E78" s="13" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="14" t="inlineStr">
-        <is>
-          <t>MS-02</t>
-        </is>
-      </c>
-      <c r="B79" s="15" t="inlineStr">
-        <is>
-          <t>Network Availability</t>
-        </is>
-      </c>
-      <c r="C79" s="16" t="inlineStr">
-        <is>
-          <t>Overall end-to-end radio and core network service availability &gt;= 99.70% monthly SLA.</t>
         </is>
       </c>
       <c r="D79" s="12" t="inlineStr"/>
       <c r="E79" s="13" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="inlineStr">
-        <is>
-          <t>MS-03</t>
-        </is>
-      </c>
-      <c r="B80" s="10" t="inlineStr">
-        <is>
-          <t>Critical Incident MTTR</t>
-        </is>
-      </c>
-      <c r="C80" s="11" t="inlineStr">
-        <is>
-          <t>Mean Time to Restore full service for Critical / Severity-1 outages: &lt;= 2hours in urban areas; &lt;= 4hours in rural areas.</t>
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>MS-02</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>Network Availability</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>Overall end-to-end radio and core network service availability &gt;= 99.70% monthly SLA.</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr"/>
       <c r="E80" s="13" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="14" t="inlineStr">
-        <is>
-          <t>MS-04</t>
-        </is>
-      </c>
-      <c r="B81" s="15" t="inlineStr">
-        <is>
-          <t>First Line Maint. (FLM)</t>
-        </is>
-      </c>
-      <c r="C81" s="16" t="inlineStr">
-        <is>
-          <t>Dedicated nationwide field dispatch teams with dedicated 4x4 vehicles, fusion splicers, OTDRs, spectrum analyzers, and climbing gear.</t>
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>MS-03</t>
+        </is>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t>Critical Incident MTTR</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="inlineStr">
+        <is>
+          <t>Mean Time to Restore full service for Critical / Severity-1 outages: &lt;= 2hours in urban areas; &lt;= 4hours in rural areas.</t>
         </is>
       </c>
       <c r="D81" s="12" t="inlineStr"/>
       <c r="E81" s="13" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="9" t="inlineStr">
-        <is>
-          <t>MS-05</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="inlineStr">
-        <is>
-          <t>Preventive Maintenance</t>
-        </is>
-      </c>
-      <c r="C82" s="11" t="inlineStr">
-        <is>
-          <t>Quarterly scheduled site inspections: Antenna bracket torque checks, RF cable weatherproofing, battery impedance tests, genset runs.</t>
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>MS-04</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>First Line Maint. (FLM)</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>Dedicated nationwide field dispatch teams with dedicated 4x4 vehicles, fusion splicers, OTDRs, spectrum analyzers, and climbing gear.</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr"/>
       <c r="E82" s="13" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="14" t="inlineStr">
-        <is>
-          <t>MS-06</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>Spare Parts Logistics</t>
-        </is>
-      </c>
-      <c r="C83" s="16" t="inlineStr">
-        <is>
-          <t>Automated SPMS maintaining regional buffer stock; guaranteed Next Business Day (NBD) hardware replacement delivery nationwide.</t>
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>MS-05</t>
+        </is>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t>Preventive Maintenance</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>Quarterly scheduled site inspections: Antenna bracket torque checks, RF cable weatherproofing, battery impedance tests, genset runs.</t>
         </is>
       </c>
       <c r="D83" s="12" t="inlineStr"/>
       <c r="E83" s="13" t="inlineStr"/>
     </row>
     <row r="84" ht="22" customHeight="1">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>MS-06</t>
+        </is>
+      </c>
+      <c r="B84" s="27" t="n"/>
+      <c r="C84" s="27" t="n"/>
+      <c r="D84" s="27" t="n"/>
+      <c r="E84" s="28" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
         <is>
           <t>SECTION 7: 5G CUSTOMER PREMISES EQUIPMENT (CPE - LOT 7)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="9" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="9" t="inlineStr">
         <is>
           <t>CPE-01</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>3GPP Standards &amp; Modes</t>
         </is>
       </c>
-      <c r="C85" s="11" t="inlineStr">
+      <c r="C86" s="11" t="inlineStr">
         <is>
           <t>3GPP Release 16/17 compliant 5G NR sub-6 GHz Standalone (SA) and Non-Standalone (NSA) operation.</t>
-        </is>
-      </c>
-      <c r="D85" s="12" t="inlineStr"/>
-      <c r="E85" s="13" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="14" t="inlineStr">
-        <is>
-          <t>CPE-02</t>
-        </is>
-      </c>
-      <c r="B86" s="15" t="inlineStr">
-        <is>
-          <t>Frequency Bands</t>
-        </is>
-      </c>
-      <c r="C86" s="16" t="inlineStr">
-        <is>
-          <t>Native Band n50 (1432 – 1517 MHz, supporting 60 MHz and 80 MHz channel bandwidths) plus fallback sub-6 GHz bands (n1, n3, n7, n28, n41, n77, n78).</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr"/>
       <c r="E86" s="13" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="9" t="inlineStr">
-        <is>
-          <t>CPE-03</t>
-        </is>
-      </c>
-      <c r="B87" s="10" t="inlineStr">
-        <is>
-          <t>Indoor CPE Antenna &amp; MIMO</t>
-        </is>
-      </c>
-      <c r="C87" s="11" t="inlineStr">
-        <is>
-          <t>High-gain omnidirectional multi-element internal antenna array (minimum &gt;= 8.0 dBi gain across Band n50); 4x4 MIMO DL, 2x2 MIMO UL.</t>
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>CPE-02</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>Frequency Bands</t>
+        </is>
+      </c>
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>Native Band n50 (1432 – 1517 MHz, supporting 60 MHz and 80 MHz channel bandwidths) plus fallback sub-6 GHz bands (n1, n3, n7, n28, n41, n77, n78).</t>
         </is>
       </c>
       <c r="D87" s="12" t="inlineStr"/>
       <c r="E87" s="13" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="14" t="inlineStr">
-        <is>
-          <t>CPE-04</t>
-        </is>
-      </c>
-      <c r="B88" s="15" t="inlineStr">
-        <is>
-          <t>Outdoor CPE Antenna &amp; MIMO</t>
-        </is>
-      </c>
-      <c r="C88" s="16" t="inlineStr">
-        <is>
-          <t>High-gain directional integrated antenna array (minimum &gt;= 12.0 dBi gain across Band n50); 4x4 MIMO DL, 2x2 MIMO UL; adjustable pole/wall mounting bracket.</t>
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>CPE-03</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>Indoor CPE Antenna &amp; MIMO</t>
+        </is>
+      </c>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t>High-gain omnidirectional multi-element internal antenna array (minimum &gt;= 8.0 dBi gain across Band n50); 4x4 MIMO DL, 2x2 MIMO UL.</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr"/>
       <c r="E88" s="13" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="9" t="inlineStr">
-        <is>
-          <t>CPE-05</t>
-        </is>
-      </c>
-      <c r="B89" s="10" t="inlineStr">
-        <is>
-          <t>Wi-Fi Subsystem</t>
-        </is>
-      </c>
-      <c r="C89" s="11" t="inlineStr">
-        <is>
-          <t>Dual-band Wi-Fi 6 (802.11ax) 2.4 GHz (2x2) and 5 GHz (2x2) concurrent, OFDMA, MU-MIMO, WPA3-Personal encryption.</t>
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>CPE-04</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>Outdoor CPE Antenna &amp; MIMO</t>
+        </is>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>High-gain directional integrated antenna array (minimum &gt;= 12.0 dBi gain across Band n50); 4x4 MIMO DL, 2x2 MIMO UL; adjustable pole/wall mounting bracket.</t>
         </is>
       </c>
       <c r="D89" s="12" t="inlineStr"/>
       <c r="E89" s="13" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="14" t="inlineStr">
-        <is>
-          <t>CPE-06</t>
-        </is>
-      </c>
-      <c r="B90" s="15" t="inlineStr">
-        <is>
-          <t>Ethernet Interfaces</t>
-        </is>
-      </c>
-      <c r="C90" s="16" t="inlineStr">
-        <is>
-          <t>Indoor CPE: Minimum 1x 2.5GE + 2x 1GE RJ-45 LAN ports. Outdoor CPE: 1x 2.5GE PoE input port plus companion indoor Wi-Fi 6 router/gateway and 802.3at PoE injector included in kit.</t>
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>CPE-05</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>Wi-Fi Subsystem</t>
+        </is>
+      </c>
+      <c r="C90" s="11" t="inlineStr">
+        <is>
+          <t>Dual-band Wi-Fi 6 (802.11ax) 2.4 GHz (2x2) and 5 GHz (2x2) concurrent, OFDMA, MU-MIMO, WPA3-Personal encryption.</t>
         </is>
       </c>
       <c r="D90" s="12" t="inlineStr"/>
       <c r="E90" s="13" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="9" t="inlineStr">
-        <is>
-          <t>CPE-07</t>
-        </is>
-      </c>
-      <c r="B91" s="10" t="inlineStr">
-        <is>
-          <t>Environmental Rating</t>
-        </is>
-      </c>
-      <c r="C91" s="11" t="inlineStr">
-        <is>
-          <t>Outdoor CPE: IP67 dust/water ingress protection, operating temperature -10°C to +55°C, 200 km/h wind survivability. Indoor CPE: IP20, 0°C to +40°C.</t>
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>CPE-06</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="inlineStr">
+        <is>
+          <t>Ethernet Interfaces</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>Indoor CPE: Minimum 1x 2.5GE + 2x 1GE RJ-45 LAN ports. Outdoor CPE: 1x 2.5GE PoE input port plus companion indoor Wi-Fi 6 router/gateway and 802.3at PoE injector included in kit.</t>
         </is>
       </c>
       <c r="D91" s="12" t="inlineStr"/>
       <c r="E91" s="13" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="14" t="inlineStr">
-        <is>
-          <t>CPE-08</t>
-        </is>
-      </c>
-      <c r="B92" s="15" t="inlineStr">
-        <is>
-          <t>Remote Device Management</t>
-        </is>
-      </c>
-      <c r="C92" s="16" t="inlineStr">
-        <is>
-          <t>Broadband Forum TR-069 and TR-369 (USP) support with complete TR-181 data model, SNMPv2/v3, and secure ACS provisioning.</t>
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>CPE-07</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Environmental Rating</t>
+        </is>
+      </c>
+      <c r="C92" s="11" t="inlineStr">
+        <is>
+          <t>Outdoor CPE: IP67 dust/water ingress protection, operating temperature -10°C to +55°C, 200 km/h wind survivability. Indoor CPE: IP20, 0°C to +40°C.</t>
         </is>
       </c>
       <c r="D92" s="12" t="inlineStr"/>
       <c r="E92" s="13" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" s="9" t="inlineStr">
-        <is>
-          <t>CPE-09</t>
-        </is>
-      </c>
-      <c r="B93" s="10" t="inlineStr">
-        <is>
-          <t>Firmware &amp; Security</t>
-        </is>
-      </c>
-      <c r="C93" s="11" t="inlineStr">
-        <is>
-          <t>Secure Boot with cryptographic signature verification, automated FOTA (Firmware-Over-The-Air) batch upgrades, and operator lock capability.</t>
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>CPE-08</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="inlineStr">
+        <is>
+          <t>Remote Device Management</t>
+        </is>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>Broadband Forum TR-069 and TR-369 (USP) support with complete TR-181 data model, SNMPv2/v3, and secure ACS provisioning.</t>
         </is>
       </c>
       <c r="D93" s="12" t="inlineStr"/>
       <c r="E93" s="13" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="14" t="inlineStr">
-        <is>
-          <t>CPE-10</t>
-        </is>
-      </c>
-      <c r="B94" s="15" t="inlineStr">
-        <is>
-          <t>SIM / eSIM Support</t>
-        </is>
-      </c>
-      <c r="C94" s="16" t="inlineStr">
-        <is>
-          <t>Standard Nano-SIM (4FF) slot with anti-theft locking cover and optional GSMA-compliant eSIM MFF2 footprint.</t>
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>CPE-09</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>Firmware &amp; Security</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>Secure Boot with cryptographic signature verification, automated FOTA (Firmware-Over-The-Air) batch upgrades, and operator lock capability.</t>
         </is>
       </c>
       <c r="D94" s="12" t="inlineStr"/>
       <c r="E94" s="13" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="9" t="inlineStr">
-        <is>
-          <t>CPE-11</t>
-        </is>
-      </c>
-      <c r="B95" s="10" t="inlineStr">
-        <is>
-          <t>Power Supply</t>
-        </is>
-      </c>
-      <c r="C95" s="11" t="inlineStr">
-        <is>
-          <t>Indoor CPE: 230V AC / 12V DC external adapter (Philippine standard Type A/B plug). Outdoor CPE: 2.5GE-capable 802.3at/bt PoE power injector and 2.5GE WAN indoor gateway companion included.</t>
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>CPE-10</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="inlineStr">
+        <is>
+          <t>SIM / eSIM Support</t>
+        </is>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>Standard Nano-SIM (4FF) slot with anti-theft locking cover and optional GSMA-compliant eSIM MFF2 footprint.</t>
         </is>
       </c>
       <c r="D95" s="12" t="inlineStr"/>
       <c r="E95" s="13" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="14" t="inlineStr">
-        <is>
-          <t>CPE-12</t>
-        </is>
-      </c>
-      <c r="B96" s="15" t="inlineStr">
-        <is>
-          <t>Certification &amp; Warranty</t>
-        </is>
-      </c>
-      <c r="C96" s="16" t="inlineStr">
-        <is>
-          <t>NTC Type Approval compliance, CE/FCC certification, and minimum 24-month hardware replacement warranty (RMA &lt;= 5 business days).</t>
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>CPE-11</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>Power Supply</t>
+        </is>
+      </c>
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>Indoor CPE: 230V AC / 12V DC external adapter (Philippine standard Type A/B plug). Outdoor CPE: 2.5GE-capable 802.3at/bt PoE power injector and 2.5GE WAN indoor gateway companion included.</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr"/>
       <c r="E96" s="13" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>CPE-12</t>
+        </is>
+      </c>
+      <c r="B97" s="15" t="inlineStr">
+        <is>
+          <t>Certification &amp; Warranty</t>
+        </is>
+      </c>
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>NTC Type Approval compliance, CE/FCC certification, and minimum 24-month hardware replacement warranty (RMA &lt;= 5 business days).</t>
+        </is>
+      </c>
+      <c r="D97" s="12" t="inlineStr"/>
+      <c r="E97" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2217,7 +2291,7 @@
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A84:E84"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A44:E44"/>
   </mergeCells>
   <dataValidations count="1">

</xml_diff>